<commit_message>
Adding use cases and business date logic for execution data
</commit_message>
<xml_diff>
--- a/KG/Batch_KG/sample_data/instance_level_data_v4.xlsx
+++ b/KG/Batch_KG/sample_data/instance_level_data_v4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Iris\practice\GenAI\code\Batch_KG\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7896BAF-516F-4249-8B06-C8B9DDF38665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22ED11AF-41D8-4BD3-8681-ADEE7EF57DC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="163">
   <si>
     <t>businessDate</t>
   </si>
@@ -522,6 +522,9 @@
   </si>
   <si>
     <t>CCAR_FS_TRIGGER</t>
+  </si>
+  <si>
+    <t>ctx_0033</t>
   </si>
 </sst>
 </file>
@@ -1155,11 +1158,11 @@
       </c>
       <c r="G2" s="13">
         <f ca="1" xml:space="preserve"> F2 + RANDBETWEEN(5, 120) / 86400</f>
-        <v>46023.264490740745</v>
+        <v>46023.264548611114</v>
       </c>
       <c r="H2" s="18">
         <f ca="1">INT((G2 - F2) * 86400/60) + MOD(INT((G2 - F2) * 86400),60)/100</f>
-        <v>0.52</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>4</v>
@@ -1187,19 +1190,19 @@
       </c>
       <c r="E3" s="13">
         <f ca="1">F3</f>
-        <v>46023.264490740745</v>
+        <v>46023.264548611114</v>
       </c>
       <c r="F3" s="13">
         <f ca="1">G2</f>
-        <v>46023.264490740745</v>
+        <v>46023.264548611114</v>
       </c>
       <c r="G3" s="13">
         <f t="shared" ref="G3:G7" ca="1" si="0" xml:space="preserve"> F3 + RANDBETWEEN(5, 120) / 86400</f>
-        <v>46023.2653587963</v>
+        <v>46023.265011574076</v>
       </c>
       <c r="H3" s="18">
         <f t="shared" ref="H3:H66" ca="1" si="1">INT((G3 - F3) * 86400/60) + MOD(INT((G3 - F3) * 86400),60)/100</f>
-        <v>1.1400000000000001</v>
+        <v>0.39</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>4</v>
@@ -1227,11 +1230,11 @@
       </c>
       <c r="E4" s="13">
         <f ca="1">F4</f>
-        <v>46023.264490740745</v>
+        <v>46023.264548611114</v>
       </c>
       <c r="F4" s="13">
         <f ca="1">G2</f>
-        <v>46023.264490740745</v>
+        <v>46023.264548611114</v>
       </c>
       <c r="G4" s="13">
         <f t="shared" ca="1" si="0"/>
@@ -1239,7 +1242,7 @@
       </c>
       <c r="H4" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>0.27</v>
+        <v>0.22</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>4</v>
@@ -1267,19 +1270,19 @@
       </c>
       <c r="E5" s="13">
         <f ca="1">F5</f>
-        <v>46023.2653587963</v>
+        <v>46023.265011574076</v>
       </c>
       <c r="F5" s="13">
         <f ca="1">G3</f>
-        <v>46023.2653587963</v>
+        <v>46023.265011574076</v>
       </c>
       <c r="G5" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46023.266342592593</v>
+        <v>46023.265949074077</v>
       </c>
       <c r="H5" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>1.24</v>
+        <v>1.21</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>4</v>
@@ -1315,11 +1318,11 @@
       </c>
       <c r="G6" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46023.265474537038</v>
+        <v>46023.265914351854</v>
       </c>
       <c r="H6" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>0.56999999999999995</v>
+        <v>1.35</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>4</v>
@@ -1347,19 +1350,19 @@
       </c>
       <c r="E7" s="13">
         <f ca="1">F7</f>
-        <v>46023.266342592593</v>
+        <v>46023.265949074077</v>
       </c>
       <c r="F7" s="13">
         <f ca="1">IF(G5 &gt; G6, G5, G6)</f>
-        <v>46023.266342592593</v>
+        <v>46023.265949074077</v>
       </c>
       <c r="G7" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46023.26766203704</v>
+        <v>46023.266250000001</v>
       </c>
       <c r="H7" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>1.54</v>
+        <v>0.25</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>4</v>
@@ -1395,7 +1398,7 @@
       </c>
       <c r="G8" s="13">
         <f ca="1" xml:space="preserve"> F8 + RANDBETWEEN(5, 120) / 86400</f>
-        <v>46024.250428240739</v>
+        <v>46024.250416666669</v>
       </c>
       <c r="H8" s="18">
         <f t="shared" ca="1" si="1"/>
@@ -1427,19 +1430,19 @@
       </c>
       <c r="E9" s="13">
         <f ca="1">F9</f>
-        <v>46024.250428240739</v>
+        <v>46024.250416666669</v>
       </c>
       <c r="F9" s="13">
         <f ca="1">G8</f>
-        <v>46024.250428240739</v>
+        <v>46024.250416666669</v>
       </c>
       <c r="G9" s="13">
         <f t="shared" ref="G9:G19" ca="1" si="2" xml:space="preserve"> F9 + RANDBETWEEN(5, 120) / 86400</f>
-        <v>46024.250960648147</v>
+        <v>46024.251180555555</v>
       </c>
       <c r="H9" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>0.46</v>
+        <v>1.05</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>4</v>
@@ -1467,19 +1470,19 @@
       </c>
       <c r="E10" s="13">
         <f t="shared" ref="E10:E13" ca="1" si="3">F10</f>
-        <v>46024.250428240739</v>
+        <v>46024.250416666669</v>
       </c>
       <c r="F10" s="13">
         <f ca="1">G8</f>
-        <v>46024.250428240739</v>
+        <v>46024.250416666669</v>
       </c>
       <c r="G10" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46024.251608796294</v>
+        <v>46024.250648148154</v>
       </c>
       <c r="H10" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>1.41</v>
+        <v>0.2</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>4</v>
@@ -1507,19 +1510,19 @@
       </c>
       <c r="E11" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46024.250960648147</v>
+        <v>46024.251180555555</v>
       </c>
       <c r="F11" s="13">
         <f ca="1">G9</f>
-        <v>46024.250960648147</v>
+        <v>46024.251180555555</v>
       </c>
       <c r="G11" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46024.25204861111</v>
+        <v>46024.252199074072</v>
       </c>
       <c r="H11" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>1.33</v>
+        <v>1.27</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>4</v>
@@ -1547,19 +1550,19 @@
       </c>
       <c r="E12" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46024.251608796294</v>
+        <v>46024.250648148154</v>
       </c>
       <c r="F12" s="13">
         <f ca="1">G10</f>
-        <v>46024.251608796294</v>
+        <v>46024.250648148154</v>
       </c>
       <c r="G12" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46024.252337962964</v>
+        <v>46024.251655092601</v>
       </c>
       <c r="H12" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>1.03</v>
+        <v>1.27</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>4</v>
@@ -1587,19 +1590,19 @@
       </c>
       <c r="E13" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46024.252337962964</v>
+        <v>46024.252199074072</v>
       </c>
       <c r="F13" s="13">
         <f ca="1">IF(G11 &gt; G12, G11, G12)</f>
-        <v>46024.252337962964</v>
+        <v>46024.252199074072</v>
       </c>
       <c r="G13" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46024.253275462965</v>
+        <v>46024.253425925926</v>
       </c>
       <c r="H13" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>1.21</v>
+        <v>1.46</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>4</v>
@@ -1635,11 +1638,11 @@
       </c>
       <c r="G14" s="13">
         <f ca="1" xml:space="preserve"> F14 + RANDBETWEEN(5, 120) / 86400</f>
-        <v>46025.250277777777</v>
+        <v>46025.250717592593</v>
       </c>
       <c r="H14" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>0.23</v>
+        <v>1.02</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>4</v>
@@ -1667,19 +1670,19 @@
       </c>
       <c r="E15" s="13">
         <f ca="1">F15</f>
-        <v>46025.250277777777</v>
+        <v>46025.250717592593</v>
       </c>
       <c r="F15" s="13">
         <f ca="1">G14</f>
-        <v>46025.250277777777</v>
+        <v>46025.250717592593</v>
       </c>
       <c r="G15" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46025.250520833331</v>
+        <v>46025.251932870371</v>
       </c>
       <c r="H15" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>0.2</v>
+        <v>1.45</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>4</v>
@@ -1707,19 +1710,19 @@
       </c>
       <c r="E16" s="13">
         <f t="shared" ref="E16:E19" ca="1" si="4">F16</f>
-        <v>46025.250277777777</v>
+        <v>46025.250717592593</v>
       </c>
       <c r="F16" s="13">
         <f ca="1">G14</f>
-        <v>46025.250277777777</v>
+        <v>46025.250717592593</v>
       </c>
       <c r="G16" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46025.251585648148</v>
+        <v>46025.251400462963</v>
       </c>
       <c r="H16" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>1.53</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>4</v>
@@ -1747,19 +1750,19 @@
       </c>
       <c r="E17" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46025.250520833331</v>
+        <v>46025.251932870371</v>
       </c>
       <c r="F17" s="13">
         <f ca="1">G15</f>
-        <v>46025.250520833331</v>
+        <v>46025.251932870371</v>
       </c>
       <c r="G17" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46025.25163194444</v>
+        <v>46025.252812500003</v>
       </c>
       <c r="H17" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>1.35</v>
+        <v>1.1599999999999999</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>4</v>
@@ -1787,19 +1790,19 @@
       </c>
       <c r="E18" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46025.251585648148</v>
+        <v>46025.251400462963</v>
       </c>
       <c r="F18" s="13">
         <f ca="1">G16</f>
-        <v>46025.251585648148</v>
+        <v>46025.251400462963</v>
       </c>
       <c r="G18" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46025.252430555556</v>
+        <v>46025.251747685186</v>
       </c>
       <c r="H18" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>1.1299999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>4</v>
@@ -1827,19 +1830,19 @@
       </c>
       <c r="E19" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46025.252430555556</v>
+        <v>46025.252812500003</v>
       </c>
       <c r="F19" s="13">
         <f ca="1">IF(G17 &gt; G18, G17, G18)</f>
-        <v>46025.252430555556</v>
+        <v>46025.252812500003</v>
       </c>
       <c r="G19" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46025.252847222226</v>
+        <v>46025.253020833334</v>
       </c>
       <c r="H19" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>0.36</v>
+        <v>0.17</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>4</v>
@@ -1875,11 +1878,11 @@
       </c>
       <c r="G20" s="13">
         <f ca="1" xml:space="preserve"> F20 + RANDBETWEEN(280, 400) / 86400</f>
-        <v>46023.587835648148</v>
+        <v>46023.586851851855</v>
       </c>
       <c r="H20" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>6.28</v>
+        <v>5.04</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>4</v>
@@ -1907,19 +1910,19 @@
       </c>
       <c r="E21" s="13">
         <f ca="1">F21</f>
-        <v>46023.587835648148</v>
+        <v>46023.586851851855</v>
       </c>
       <c r="F21" s="13">
         <f ca="1">G20</f>
-        <v>46023.587835648148</v>
+        <v>46023.586851851855</v>
       </c>
       <c r="G21" s="13">
         <f ca="1" xml:space="preserve"> F21 + RANDBETWEEN(280, 390) / 86400</f>
-        <v>46023.591157407405</v>
+        <v>46023.590196759265</v>
       </c>
       <c r="H21" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>4.46</v>
+        <v>4.49</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>4</v>
@@ -1947,19 +1950,19 @@
       </c>
       <c r="E22" s="13">
         <f t="shared" ref="E22:E28" ca="1" si="5">F22</f>
-        <v>46023.587835648148</v>
+        <v>46023.586851851855</v>
       </c>
       <c r="F22" s="13">
         <f ca="1">G20</f>
-        <v>46023.587835648148</v>
+        <v>46023.586851851855</v>
       </c>
       <c r="G22" s="13">
         <f ca="1" xml:space="preserve"> F22 + RANDBETWEEN(350, 450) / 86400</f>
-        <v>46023.592372685183</v>
+        <v>46023.591238425928</v>
       </c>
       <c r="H22" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>6.31</v>
+        <v>6.18</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>4</v>
@@ -1987,19 +1990,19 @@
       </c>
       <c r="E23" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46023.591157407405</v>
+        <v>46023.590196759265</v>
       </c>
       <c r="F23" s="13">
         <f ca="1">G21</f>
-        <v>46023.591157407405</v>
+        <v>46023.590196759265</v>
       </c>
       <c r="G23" s="13">
         <f ca="1" xml:space="preserve"> F23 + RANDBETWEEN(410, 710) / 86400</f>
-        <v>46023.596840277773</v>
+        <v>46023.597546296303</v>
       </c>
       <c r="H23" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>8.1</v>
+        <v>10.35</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>4</v>
@@ -2027,19 +2030,19 @@
       </c>
       <c r="E24" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46023.592372685183</v>
+        <v>46023.591238425928</v>
       </c>
       <c r="F24" s="13">
         <f ca="1">G22</f>
-        <v>46023.592372685183</v>
+        <v>46023.591238425928</v>
       </c>
       <c r="G24" s="13">
         <f ca="1" xml:space="preserve"> F24 + RANDBETWEEN(350, 650) / 86400</f>
-        <v>46023.597928240742</v>
+        <v>46023.595451388894</v>
       </c>
       <c r="H24" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>8</v>
+        <v>6.04</v>
       </c>
       <c r="I24" s="3" t="s">
         <v>4</v>
@@ -2067,19 +2070,19 @@
       </c>
       <c r="E25" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46023.596840277773</v>
+        <v>46023.597546296303</v>
       </c>
       <c r="F25" s="13">
         <f ca="1">G23</f>
-        <v>46023.596840277773</v>
+        <v>46023.597546296303</v>
       </c>
       <c r="G25" s="13">
         <f ca="1" xml:space="preserve"> F25 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46023.601898148147</v>
+        <v>46023.602002314823</v>
       </c>
       <c r="H25" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>7.17</v>
+        <v>6.25</v>
       </c>
       <c r="I25" s="3" t="s">
         <v>4</v>
@@ -2107,19 +2110,19 @@
       </c>
       <c r="E26" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46023.597928240742</v>
+        <v>46023.595451388894</v>
       </c>
       <c r="F26" s="13">
         <f ca="1">G24</f>
-        <v>46023.597928240742</v>
+        <v>46023.595451388894</v>
       </c>
       <c r="G26" s="13">
         <f ca="1" xml:space="preserve"> F26 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46023.601979166669</v>
+        <v>46023.599479166674</v>
       </c>
       <c r="H26" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>5.5</v>
+        <v>5.48</v>
       </c>
       <c r="I26" s="3" t="s">
         <v>4</v>
@@ -2147,19 +2150,19 @@
       </c>
       <c r="E27" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46023.601979166669</v>
+        <v>46023.599479166674</v>
       </c>
       <c r="F27" s="13">
         <f ca="1">G26</f>
-        <v>46023.601979166669</v>
+        <v>46023.599479166674</v>
       </c>
       <c r="G27" s="13">
         <f ca="1" xml:space="preserve"> F27 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46023.604988425926</v>
+        <v>46023.603101851862</v>
       </c>
       <c r="H27" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>4.1900000000000004</v>
+        <v>5.13</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>4</v>
@@ -2187,19 +2190,19 @@
       </c>
       <c r="E28" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46023.604988425926</v>
+        <v>46023.603101851862</v>
       </c>
       <c r="F28" s="13">
         <f ca="1">IF(G25 &gt; G27, G25, G27)</f>
-        <v>46023.604988425926</v>
+        <v>46023.603101851862</v>
       </c>
       <c r="G28" s="13">
         <f ca="1" xml:space="preserve"> F28 + RANDBETWEEN(150, 350) / 86400</f>
-        <v>46023.606724537036</v>
+        <v>46023.606226851865</v>
       </c>
       <c r="H28" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>2.29</v>
+        <v>4.3</v>
       </c>
       <c r="I28" s="3" t="s">
         <v>4</v>
@@ -2235,11 +2238,11 @@
       </c>
       <c r="G29" s="13">
         <f ca="1" xml:space="preserve"> F29 + RANDBETWEEN(280, 400) / 86400</f>
-        <v>46024.58729166667</v>
+        <v>46024.587800925925</v>
       </c>
       <c r="H29" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>5.42</v>
+        <v>6.25</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>4</v>
@@ -2267,19 +2270,19 @@
       </c>
       <c r="E30" s="13">
         <f ca="1">F30</f>
-        <v>46024.58729166667</v>
+        <v>46024.587800925925</v>
       </c>
       <c r="F30" s="13">
         <f ca="1">G29</f>
-        <v>46024.58729166667</v>
+        <v>46024.587800925925</v>
       </c>
       <c r="G30" s="13">
         <f ca="1" xml:space="preserve"> F30 + RANDBETWEEN(280, 390) / 86400</f>
-        <v>46024.591562500005</v>
+        <v>46024.591770833329</v>
       </c>
       <c r="H30" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>6.09</v>
+        <v>5.42</v>
       </c>
       <c r="I30" s="3" t="s">
         <v>4</v>
@@ -2307,19 +2310,19 @@
       </c>
       <c r="E31" s="13">
         <f t="shared" ref="E31:E37" ca="1" si="6">F31</f>
-        <v>46024.58729166667</v>
+        <v>46024.587800925925</v>
       </c>
       <c r="F31" s="13">
         <f ca="1">G29</f>
-        <v>46024.58729166667</v>
+        <v>46024.587800925925</v>
       </c>
       <c r="G31" s="13">
         <f ca="1" xml:space="preserve"> F31 + RANDBETWEEN(350, 450) / 86400</f>
-        <v>46024.592106481483</v>
+        <v>46024.592199074075</v>
       </c>
       <c r="H31" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>6.55</v>
+        <v>6.2</v>
       </c>
       <c r="I31" s="3" t="s">
         <v>4</v>
@@ -2347,19 +2350,19 @@
       </c>
       <c r="E32" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46024.591562500005</v>
+        <v>46024.591770833329</v>
       </c>
       <c r="F32" s="13">
         <f ca="1">G30</f>
-        <v>46024.591562500005</v>
+        <v>46024.591770833329</v>
       </c>
       <c r="G32" s="13">
         <f ca="1" xml:space="preserve"> F32 + RANDBETWEEN(410, 710) / 86400</f>
-        <v>46024.598333333335</v>
+        <v>46024.599583333329</v>
       </c>
       <c r="H32" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>9.44</v>
+        <v>11.15</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>4</v>
@@ -2387,19 +2390,19 @@
       </c>
       <c r="E33" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46024.592106481483</v>
+        <v>46024.592199074075</v>
       </c>
       <c r="F33" s="13">
         <f ca="1">G31</f>
-        <v>46024.592106481483</v>
+        <v>46024.592199074075</v>
       </c>
       <c r="G33" s="13">
         <f ca="1" xml:space="preserve"> F33 + RANDBETWEEN(350, 650) / 86400</f>
-        <v>46024.598483796297</v>
+        <v>46024.597037037041</v>
       </c>
       <c r="H33" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>9.1</v>
+        <v>6.58</v>
       </c>
       <c r="I33" s="3" t="s">
         <v>4</v>
@@ -2427,19 +2430,19 @@
       </c>
       <c r="E34" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46024.598333333335</v>
+        <v>46024.599583333329</v>
       </c>
       <c r="F34" s="13">
         <f ca="1">G32</f>
-        <v>46024.598333333335</v>
+        <v>46024.599583333329</v>
       </c>
       <c r="G34" s="13">
         <f ca="1" xml:space="preserve"> F34 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46024.602314814816</v>
+        <v>46024.604224537034</v>
       </c>
       <c r="H34" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>5.43</v>
+        <v>6.41</v>
       </c>
       <c r="I34" s="3" t="s">
         <v>4</v>
@@ -2467,19 +2470,19 @@
       </c>
       <c r="E35" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46024.598483796297</v>
+        <v>46024.597037037041</v>
       </c>
       <c r="F35" s="13">
         <f ca="1">G33</f>
-        <v>46024.598483796297</v>
+        <v>46024.597037037041</v>
       </c>
       <c r="G35" s="13">
         <f ca="1" xml:space="preserve"> F35 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46024.601701388892</v>
+        <v>46024.60128472223</v>
       </c>
       <c r="H35" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>4.38</v>
+        <v>6.07</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>4</v>
@@ -2507,19 +2510,19 @@
       </c>
       <c r="E36" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46024.601701388892</v>
+        <v>46024.60128472223</v>
       </c>
       <c r="F36" s="13">
         <f ca="1">G35</f>
-        <v>46024.601701388892</v>
+        <v>46024.60128472223</v>
       </c>
       <c r="G36" s="13">
         <f ca="1" xml:space="preserve"> F36 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46024.605162037042</v>
+        <v>46024.604780092603</v>
       </c>
       <c r="H36" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>4.59</v>
+        <v>5.0199999999999996</v>
       </c>
       <c r="I36" s="3" t="s">
         <v>4</v>
@@ -2547,19 +2550,19 @@
       </c>
       <c r="E37" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46024.605162037042</v>
+        <v>46024.604780092603</v>
       </c>
       <c r="F37" s="13">
         <f ca="1">IF(G34 &gt; G36, G34, G36)</f>
-        <v>46024.605162037042</v>
+        <v>46024.604780092603</v>
       </c>
       <c r="G37" s="13">
         <f ca="1" xml:space="preserve"> F37 + RANDBETWEEN(150, 350) / 86400</f>
-        <v>46024.609062500007</v>
+        <v>46024.607013888897</v>
       </c>
       <c r="H37" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>5.37</v>
+        <v>3.12</v>
       </c>
       <c r="I37" s="3" t="s">
         <v>4</v>
@@ -2595,11 +2598,11 @@
       </c>
       <c r="G38" s="13">
         <f ca="1" xml:space="preserve"> F38 + RANDBETWEEN(280, 400) / 86400</f>
-        <v>46025.587754629632</v>
+        <v>46025.586678240747</v>
       </c>
       <c r="H38" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>6.22</v>
+        <v>4.49</v>
       </c>
       <c r="I38" s="3" t="s">
         <v>4</v>
@@ -2627,19 +2630,19 @@
       </c>
       <c r="E39" s="13">
         <f ca="1">F39</f>
-        <v>46025.587754629632</v>
+        <v>46025.586678240747</v>
       </c>
       <c r="F39" s="13">
         <f ca="1">G38</f>
-        <v>46025.587754629632</v>
+        <v>46025.586678240747</v>
       </c>
       <c r="G39" s="13">
         <f ca="1" xml:space="preserve"> F39 + RANDBETWEEN(280, 390) / 86400</f>
-        <v>46025.591793981483</v>
+        <v>46025.590949074081</v>
       </c>
       <c r="H39" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>5.48</v>
+        <v>6.09</v>
       </c>
       <c r="I39" s="3" t="s">
         <v>4</v>
@@ -2667,19 +2670,19 @@
       </c>
       <c r="E40" s="13">
         <f t="shared" ref="E40:E46" ca="1" si="7">F40</f>
-        <v>46025.587754629632</v>
+        <v>46025.586678240747</v>
       </c>
       <c r="F40" s="13">
         <f ca="1">G38</f>
-        <v>46025.587754629632</v>
+        <v>46025.586678240747</v>
       </c>
       <c r="G40" s="13">
         <f ca="1" xml:space="preserve"> F40 + RANDBETWEEN(350, 450) / 86400</f>
-        <v>46025.592708333337</v>
+        <v>46025.591805555559</v>
       </c>
       <c r="H40" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>7.08</v>
+        <v>7.22</v>
       </c>
       <c r="I40" s="3" t="s">
         <v>4</v>
@@ -2707,19 +2710,19 @@
       </c>
       <c r="E41" s="13">
         <f t="shared" ca="1" si="7"/>
-        <v>46025.591793981483</v>
+        <v>46025.590949074081</v>
       </c>
       <c r="F41" s="13">
         <f ca="1">G39</f>
-        <v>46025.591793981483</v>
+        <v>46025.590949074081</v>
       </c>
       <c r="G41" s="13">
         <f ca="1" xml:space="preserve"> F41 + RANDBETWEEN(410, 710) / 86400</f>
-        <v>46025.597638888888</v>
+        <v>46025.59756944445</v>
       </c>
       <c r="H41" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>8.24</v>
+        <v>9.31</v>
       </c>
       <c r="I41" s="3" t="s">
         <v>4</v>
@@ -2747,19 +2750,19 @@
       </c>
       <c r="E42" s="13">
         <f t="shared" ca="1" si="7"/>
-        <v>46025.592708333337</v>
+        <v>46025.591805555559</v>
       </c>
       <c r="F42" s="13">
         <f ca="1">G40</f>
-        <v>46025.592708333337</v>
+        <v>46025.591805555559</v>
       </c>
       <c r="G42" s="13">
         <f ca="1" xml:space="preserve"> F42 + RANDBETWEEN(350, 650) / 86400</f>
-        <v>46025.59888888889</v>
+        <v>46025.596122685187</v>
       </c>
       <c r="H42" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>8.5299999999999994</v>
+        <v>6.12</v>
       </c>
       <c r="I42" s="3" t="s">
         <v>4</v>
@@ -2787,19 +2790,19 @@
       </c>
       <c r="E43" s="13">
         <f t="shared" ca="1" si="7"/>
-        <v>46025.597638888888</v>
+        <v>46025.59756944445</v>
       </c>
       <c r="F43" s="13">
         <f ca="1">G41</f>
-        <v>46025.597638888888</v>
+        <v>46025.59756944445</v>
       </c>
       <c r="G43" s="13">
         <f ca="1" xml:space="preserve"> F43 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46025.602152777778</v>
+        <v>46025.601331018523</v>
       </c>
       <c r="H43" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>6.3</v>
+        <v>5.24</v>
       </c>
       <c r="I43" s="3" t="s">
         <v>4</v>
@@ -2827,19 +2830,19 @@
       </c>
       <c r="E44" s="13">
         <f t="shared" ca="1" si="7"/>
-        <v>46025.59888888889</v>
+        <v>46025.596122685187</v>
       </c>
       <c r="F44" s="13">
         <f ca="1">G42</f>
-        <v>46025.59888888889</v>
+        <v>46025.596122685187</v>
       </c>
       <c r="G44" s="13">
         <f ca="1" xml:space="preserve"> F44 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46025.602951388886</v>
+        <v>46025.600590277776</v>
       </c>
       <c r="H44" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>5.5</v>
+        <v>6.25</v>
       </c>
       <c r="I44" s="3" t="s">
         <v>4</v>
@@ -2867,19 +2870,19 @@
       </c>
       <c r="E45" s="13">
         <f t="shared" ca="1" si="7"/>
-        <v>46025.602951388886</v>
+        <v>46025.600590277776</v>
       </c>
       <c r="F45" s="13">
         <f ca="1">G44</f>
-        <v>46025.602951388886</v>
+        <v>46025.600590277776</v>
       </c>
       <c r="G45" s="13">
         <f ca="1" xml:space="preserve"> F45 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46025.607928240737</v>
+        <v>46025.604780092588</v>
       </c>
       <c r="H45" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>7.09</v>
+        <v>6.01</v>
       </c>
       <c r="I45" s="3" t="s">
         <v>4</v>
@@ -2907,19 +2910,19 @@
       </c>
       <c r="E46" s="13">
         <f t="shared" ca="1" si="7"/>
-        <v>46025.607928240737</v>
+        <v>46025.604780092588</v>
       </c>
       <c r="F46" s="13">
         <f ca="1">IF(G43 &gt; G45, G43, G45)</f>
-        <v>46025.607928240737</v>
+        <v>46025.604780092588</v>
       </c>
       <c r="G46" s="13">
         <f ca="1" xml:space="preserve"> F46 + RANDBETWEEN(150, 350) / 86400</f>
-        <v>46025.610243055555</v>
+        <v>46025.607997685183</v>
       </c>
       <c r="H46" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>3.2</v>
+        <v>4.38</v>
       </c>
       <c r="I46" s="3" t="s">
         <v>4</v>
@@ -2955,11 +2958,11 @@
       </c>
       <c r="G47" s="13">
         <f ca="1" xml:space="preserve"> F47 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46023.878275462965</v>
+        <v>46023.879780092589</v>
       </c>
       <c r="H47" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>4.43</v>
+        <v>6.52</v>
       </c>
       <c r="I47" s="3" t="s">
         <v>4</v>
@@ -2987,19 +2990,19 @@
       </c>
       <c r="E48" s="13">
         <f ca="1">F48</f>
-        <v>46023.878275462965</v>
+        <v>46023.879780092589</v>
       </c>
       <c r="F48" s="13">
         <f ca="1">G47</f>
-        <v>46023.878275462965</v>
+        <v>46023.879780092589</v>
       </c>
       <c r="G48" s="13">
         <f t="shared" ref="G48:G73" ca="1" si="8" xml:space="preserve"> F48 + RANDBETWEEN(150, 350) / 86400</f>
-        <v>46023.882210648153</v>
+        <v>46023.882361111107</v>
       </c>
       <c r="H48" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>5.4</v>
+        <v>3.42</v>
       </c>
       <c r="I48" s="3" t="s">
         <v>4</v>
@@ -3027,19 +3030,19 @@
       </c>
       <c r="E49" s="13">
         <f t="shared" ref="E49:E55" ca="1" si="9">F49</f>
-        <v>46023.878275462965</v>
+        <v>46023.879780092589</v>
       </c>
       <c r="F49" s="13">
         <f ca="1">G47</f>
-        <v>46023.878275462965</v>
+        <v>46023.879780092589</v>
       </c>
       <c r="G49" s="13">
         <f ca="1" xml:space="preserve"> F49 + RANDBETWEEN(300, 500) / 86400</f>
-        <v>46023.88212962963</v>
+        <v>46023.884895833333</v>
       </c>
       <c r="H49" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>5.32</v>
+        <v>7.22</v>
       </c>
       <c r="I49" s="3" t="s">
         <v>4</v>
@@ -3067,19 +3070,19 @@
       </c>
       <c r="E50" s="13">
         <f ca="1">IF(G48 &gt; G49, G48, G49)</f>
-        <v>46023.882210648153</v>
+        <v>46023.884895833333</v>
       </c>
       <c r="F50" s="13">
         <f ca="1">IF((IF(G48 &gt; G49, G48, G49)) &gt; ResourceAvailabilityEvents!D17, (IF(G48 &gt; G49, G48, G49)), ResourceAvailabilityEvents!D17)</f>
-        <v>46023.882210648153</v>
+        <v>46023.884895833333</v>
       </c>
       <c r="G50" s="13">
         <f ca="1" xml:space="preserve"> F50 + RANDBETWEEN(450, 750) / 86400</f>
-        <v>46023.889456018522</v>
+        <v>46023.890451388892</v>
       </c>
       <c r="H50" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>10.25</v>
+        <v>8</v>
       </c>
       <c r="I50" s="3" t="s">
         <v>4</v>
@@ -3107,19 +3110,19 @@
       </c>
       <c r="E51" s="13">
         <f t="shared" ca="1" si="9"/>
-        <v>46023.889456018522</v>
+        <v>46023.890451388892</v>
       </c>
       <c r="F51" s="13">
         <f ca="1">G50</f>
-        <v>46023.889456018522</v>
+        <v>46023.890451388892</v>
       </c>
       <c r="G51" s="13">
         <f ca="1" xml:space="preserve"> F51 + RANDBETWEEN(450, 750) / 86400</f>
-        <v>46023.896192129636</v>
+        <v>46023.898900462969</v>
       </c>
       <c r="H51" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>9.42</v>
+        <v>12.1</v>
       </c>
       <c r="I51" s="3" t="s">
         <v>4</v>
@@ -3147,19 +3150,19 @@
       </c>
       <c r="E52" s="13">
         <f t="shared" ca="1" si="9"/>
-        <v>46023.896192129636</v>
+        <v>46023.898900462969</v>
       </c>
       <c r="F52" s="13">
         <f t="shared" ref="F52:F55" ca="1" si="10">G51</f>
-        <v>46023.896192129636</v>
+        <v>46023.898900462969</v>
       </c>
       <c r="G52" s="13">
         <f ca="1" xml:space="preserve"> F52 + RANDBETWEEN(200, 400) / 86400</f>
-        <v>46023.899062500008</v>
+        <v>46023.902291666673</v>
       </c>
       <c r="H52" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>4.08</v>
+        <v>4.5199999999999996</v>
       </c>
       <c r="I52" s="3" t="s">
         <v>4</v>
@@ -3187,19 +3190,19 @@
       </c>
       <c r="E53" s="13">
         <f t="shared" ca="1" si="9"/>
-        <v>46023.899062500008</v>
+        <v>46023.902291666673</v>
       </c>
       <c r="F53" s="13">
         <f t="shared" ca="1" si="10"/>
-        <v>46023.899062500008</v>
+        <v>46023.902291666673</v>
       </c>
       <c r="G53" s="13">
         <f ca="1" xml:space="preserve"> F53 + RANDBETWEEN(200, 400) / 86400</f>
-        <v>46023.901423611118</v>
+        <v>46023.905694444453</v>
       </c>
       <c r="H53" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>3.23</v>
+        <v>4.54</v>
       </c>
       <c r="I53" s="3" t="s">
         <v>4</v>
@@ -3227,19 +3230,19 @@
       </c>
       <c r="E54" s="13">
         <f t="shared" ca="1" si="9"/>
-        <v>46023.901423611118</v>
+        <v>46023.905694444453</v>
       </c>
       <c r="F54" s="13">
         <f t="shared" ca="1" si="10"/>
-        <v>46023.901423611118</v>
+        <v>46023.905694444453</v>
       </c>
       <c r="G54" s="13">
         <f ca="1" xml:space="preserve"> F54 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46023.906157407415</v>
+        <v>46023.909594907418</v>
       </c>
       <c r="H54" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>6.49</v>
+        <v>5.37</v>
       </c>
       <c r="I54" s="3" t="s">
         <v>4</v>
@@ -3267,19 +3270,19 @@
       </c>
       <c r="E55" s="13">
         <f t="shared" ca="1" si="9"/>
-        <v>46023.906157407415</v>
+        <v>46023.909594907418</v>
       </c>
       <c r="F55" s="13">
         <f t="shared" ca="1" si="10"/>
-        <v>46023.906157407415</v>
+        <v>46023.909594907418</v>
       </c>
       <c r="G55" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46023.909826388895</v>
+        <v>46023.912719907421</v>
       </c>
       <c r="H55" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>5.16</v>
+        <v>4.3</v>
       </c>
       <c r="I55" s="3" t="s">
         <v>4</v>
@@ -3315,11 +3318,11 @@
       </c>
       <c r="G56" s="13">
         <f ca="1" xml:space="preserve"> F56 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46024.879050925927</v>
+        <v>46024.879629629628</v>
       </c>
       <c r="H56" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>5.5</v>
+        <v>6.39</v>
       </c>
       <c r="I56" s="3" t="s">
         <v>4</v>
@@ -3347,19 +3350,19 @@
       </c>
       <c r="E57" s="13">
         <f ca="1">F57</f>
-        <v>46024.879050925927</v>
+        <v>46024.879629629628</v>
       </c>
       <c r="F57" s="13">
         <f ca="1">G56</f>
-        <v>46024.879050925927</v>
+        <v>46024.879629629628</v>
       </c>
       <c r="G57" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46024.881388888891</v>
+        <v>46024.883171296293</v>
       </c>
       <c r="H57" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>3.22</v>
+        <v>5.05</v>
       </c>
       <c r="I57" s="3" t="s">
         <v>4</v>
@@ -3387,19 +3390,19 @@
       </c>
       <c r="E58" s="13">
         <f t="shared" ref="E58:E64" ca="1" si="11">F58</f>
-        <v>46024.879050925927</v>
+        <v>46024.879629629628</v>
       </c>
       <c r="F58" s="13">
         <f ca="1">G56</f>
-        <v>46024.879050925927</v>
+        <v>46024.879629629628</v>
       </c>
       <c r="G58" s="13">
         <f ca="1" xml:space="preserve"> F58 + RANDBETWEEN(300, 500) / 86400</f>
-        <v>46024.883414351854</v>
+        <v>46024.88381944444</v>
       </c>
       <c r="H58" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>6.17</v>
+        <v>6.01</v>
       </c>
       <c r="I58" s="3" t="s">
         <v>4</v>
@@ -3427,19 +3430,19 @@
       </c>
       <c r="E59" s="13">
         <f ca="1">IF(G57 &gt; G58, G57, G58)</f>
-        <v>46024.883414351854</v>
+        <v>46024.88381944444</v>
       </c>
       <c r="F59" s="13">
         <f ca="1">IF((IF(G57 &gt; G58, G57, G58)) &gt; ResourceAvailabilityEvents!D18, (IF(G57 &gt; G58, G57, G58)), ResourceAvailabilityEvents!D18)</f>
-        <v>46024.883414351854</v>
+        <v>46024.88381944444</v>
       </c>
       <c r="G59" s="13">
         <f ca="1" xml:space="preserve"> F59 + RANDBETWEEN(450, 750) / 86400</f>
-        <v>46024.891388888893</v>
+        <v>46024.890787037031</v>
       </c>
       <c r="H59" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>11.29</v>
+        <v>10.01</v>
       </c>
       <c r="I59" s="3" t="s">
         <v>4</v>
@@ -3467,19 +3470,19 @@
       </c>
       <c r="E60" s="13">
         <f t="shared" ca="1" si="11"/>
-        <v>46024.891388888893</v>
+        <v>46024.890787037031</v>
       </c>
       <c r="F60" s="13">
         <f ca="1">G59</f>
-        <v>46024.891388888893</v>
+        <v>46024.890787037031</v>
       </c>
       <c r="G60" s="13">
         <f ca="1" xml:space="preserve"> F60 + RANDBETWEEN(450, 750) / 86400</f>
-        <v>46024.898703703708</v>
+        <v>46024.897453703699</v>
       </c>
       <c r="H60" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>10.32</v>
+        <v>9.36</v>
       </c>
       <c r="I60" s="3" t="s">
         <v>4</v>
@@ -3507,19 +3510,19 @@
       </c>
       <c r="E61" s="13">
         <f t="shared" ca="1" si="11"/>
-        <v>46024.898703703708</v>
+        <v>46024.897453703699</v>
       </c>
       <c r="F61" s="13">
         <f t="shared" ref="F61:F64" ca="1" si="12">G60</f>
-        <v>46024.898703703708</v>
+        <v>46024.897453703699</v>
       </c>
       <c r="G61" s="13">
         <f ca="1" xml:space="preserve"> F61 + RANDBETWEEN(200, 400) / 86400</f>
-        <v>46024.901018518525</v>
+        <v>46024.900891203702</v>
       </c>
       <c r="H61" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>3.2</v>
+        <v>4.57</v>
       </c>
       <c r="I61" s="3" t="s">
         <v>4</v>
@@ -3547,19 +3550,19 @@
       </c>
       <c r="E62" s="13">
         <f t="shared" ca="1" si="11"/>
-        <v>46024.901018518525</v>
+        <v>46024.900891203702</v>
       </c>
       <c r="F62" s="13">
         <f t="shared" ca="1" si="12"/>
-        <v>46024.901018518525</v>
+        <v>46024.900891203702</v>
       </c>
       <c r="G62" s="13">
         <f ca="1" xml:space="preserve"> F62 + RANDBETWEEN(200, 400) / 86400</f>
-        <v>46024.904907407414</v>
+        <v>46024.905497685184</v>
       </c>
       <c r="H62" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>5.35</v>
+        <v>6.37</v>
       </c>
       <c r="I62" s="3" t="s">
         <v>4</v>
@@ -3587,19 +3590,19 @@
       </c>
       <c r="E63" s="13">
         <f t="shared" ca="1" si="11"/>
-        <v>46024.904907407414</v>
+        <v>46024.905497685184</v>
       </c>
       <c r="F63" s="13">
         <f t="shared" ca="1" si="12"/>
-        <v>46024.904907407414</v>
+        <v>46024.905497685184</v>
       </c>
       <c r="G63" s="13">
         <f ca="1" xml:space="preserve"> F63 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46024.908252314824</v>
+        <v>46024.908518518518</v>
       </c>
       <c r="H63" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>4.49</v>
+        <v>4.21</v>
       </c>
       <c r="I63" s="3" t="s">
         <v>4</v>
@@ -3627,19 +3630,19 @@
       </c>
       <c r="E64" s="13">
         <f t="shared" ca="1" si="11"/>
-        <v>46024.908252314824</v>
+        <v>46024.908518518518</v>
       </c>
       <c r="F64" s="13">
         <f t="shared" ca="1" si="12"/>
-        <v>46024.908252314824</v>
+        <v>46024.908518518518</v>
       </c>
       <c r="G64" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46024.911134259266</v>
+        <v>46024.910277777773</v>
       </c>
       <c r="H64" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>4.08</v>
+        <v>2.31</v>
       </c>
       <c r="I64" s="3" t="s">
         <v>4</v>
@@ -3675,11 +3678,11 @@
       </c>
       <c r="G65" s="13">
         <f ca="1" xml:space="preserve"> F65 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46025.879560185182</v>
+        <v>46025.879918981482</v>
       </c>
       <c r="H65" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>6.33</v>
+        <v>7.05</v>
       </c>
       <c r="I65" s="3" t="s">
         <v>4</v>
@@ -3707,19 +3710,19 @@
       </c>
       <c r="E66" s="13">
         <f ca="1">F66</f>
-        <v>46025.879560185182</v>
+        <v>46025.879918981482</v>
       </c>
       <c r="F66" s="13">
         <f ca="1">G65</f>
-        <v>46025.879560185182</v>
+        <v>46025.879918981482</v>
       </c>
       <c r="G66" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46025.883460648147</v>
+        <v>46025.883032407408</v>
       </c>
       <c r="H66" s="18">
         <f t="shared" ca="1" si="1"/>
-        <v>5.37</v>
+        <v>4.29</v>
       </c>
       <c r="I66" s="3" t="s">
         <v>4</v>
@@ -3747,19 +3750,19 @@
       </c>
       <c r="E67" s="13">
         <f t="shared" ref="E67:E73" ca="1" si="13">F67</f>
-        <v>46025.879560185182</v>
+        <v>46025.879918981482</v>
       </c>
       <c r="F67" s="13">
         <f ca="1">G65</f>
-        <v>46025.879560185182</v>
+        <v>46025.879918981482</v>
       </c>
       <c r="G67" s="13">
         <f ca="1" xml:space="preserve"> F67 + RANDBETWEEN(300, 500) / 86400</f>
-        <v>46025.883576388886</v>
+        <v>46025.883784722224</v>
       </c>
       <c r="H67" s="18">
         <f t="shared" ref="H67:H74" ca="1" si="14">INT((G67 - F67) * 86400/60) + MOD(INT((G67 - F67) * 86400),60)/100</f>
-        <v>5.47</v>
+        <v>5.34</v>
       </c>
       <c r="I67" s="3" t="s">
         <v>4</v>
@@ -3787,19 +3790,19 @@
       </c>
       <c r="E68" s="13">
         <f ca="1">IF(G66 &gt; G67, G66, G67)</f>
-        <v>46025.883576388886</v>
+        <v>46025.883784722224</v>
       </c>
       <c r="F68" s="13">
         <f ca="1">IF((IF(G66 &gt; G67, G66, G67)) &gt; ResourceAvailabilityEvents!D19, (IF(G66 &gt; G67, G66, G67)), ResourceAvailabilityEvents!D19)</f>
-        <v>46025.883576388886</v>
+        <v>46025.883784722224</v>
       </c>
       <c r="G68" s="13">
         <f ca="1" xml:space="preserve"> F68 + RANDBETWEEN(450, 750) / 86400</f>
-        <v>46025.888969907406</v>
+        <v>46025.890208333338</v>
       </c>
       <c r="H68" s="18">
         <f t="shared" ca="1" si="14"/>
-        <v>7.46</v>
+        <v>9.15</v>
       </c>
       <c r="I68" s="3" t="s">
         <v>4</v>
@@ -3827,19 +3830,19 @@
       </c>
       <c r="E69" s="13">
         <f t="shared" ca="1" si="13"/>
-        <v>46025.888969907406</v>
+        <v>46025.890208333338</v>
       </c>
       <c r="F69" s="13">
         <f ca="1">G68</f>
-        <v>46025.888969907406</v>
+        <v>46025.890208333338</v>
       </c>
       <c r="G69" s="13">
         <f ca="1" xml:space="preserve"> F69 + RANDBETWEEN(450, 750) / 86400</f>
-        <v>46025.895439814813</v>
+        <v>46025.898252314822</v>
       </c>
       <c r="H69" s="18">
         <f t="shared" ca="1" si="14"/>
-        <v>9.18</v>
+        <v>11.35</v>
       </c>
       <c r="I69" s="3" t="s">
         <v>4</v>
@@ -3867,19 +3870,19 @@
       </c>
       <c r="E70" s="13">
         <f t="shared" ca="1" si="13"/>
-        <v>46025.895439814813</v>
+        <v>46025.898252314822</v>
       </c>
       <c r="F70" s="13">
         <f t="shared" ref="F70:F73" ca="1" si="15">G69</f>
-        <v>46025.895439814813</v>
+        <v>46025.898252314822</v>
       </c>
       <c r="G70" s="13">
         <f ca="1" xml:space="preserve"> F70 + RANDBETWEEN(200, 400) / 86400</f>
-        <v>46025.899988425925</v>
+        <v>46025.902534722227</v>
       </c>
       <c r="H70" s="18">
         <f t="shared" ca="1" si="14"/>
-        <v>6.33</v>
+        <v>6.09</v>
       </c>
       <c r="I70" s="3" t="s">
         <v>4</v>
@@ -3907,19 +3910,19 @@
       </c>
       <c r="E71" s="13">
         <f t="shared" ca="1" si="13"/>
-        <v>46025.899988425925</v>
+        <v>46025.902534722227</v>
       </c>
       <c r="F71" s="13">
         <f t="shared" ca="1" si="15"/>
-        <v>46025.899988425925</v>
+        <v>46025.902534722227</v>
       </c>
       <c r="G71" s="13">
         <f ca="1" xml:space="preserve"> F71 + RANDBETWEEN(200, 400) / 86400</f>
-        <v>46025.902997685182</v>
+        <v>46025.907141203708</v>
       </c>
       <c r="H71" s="18">
         <f t="shared" ca="1" si="14"/>
-        <v>4.1900000000000004</v>
+        <v>6.37</v>
       </c>
       <c r="I71" s="3" t="s">
         <v>4</v>
@@ -3947,19 +3950,19 @@
       </c>
       <c r="E72" s="13">
         <f t="shared" ca="1" si="13"/>
-        <v>46025.902997685182</v>
+        <v>46025.907141203708</v>
       </c>
       <c r="F72" s="13">
         <f t="shared" ca="1" si="15"/>
-        <v>46025.902997685182</v>
+        <v>46025.907141203708</v>
       </c>
       <c r="G72" s="13">
         <f ca="1" xml:space="preserve"> F72 + RANDBETWEEN(250, 450) / 86400</f>
-        <v>46025.90693287037</v>
+        <v>46025.910277777781</v>
       </c>
       <c r="H72" s="18">
         <f t="shared" ca="1" si="14"/>
-        <v>5.4</v>
+        <v>4.3</v>
       </c>
       <c r="I72" s="3" t="s">
         <v>4</v>
@@ -3987,19 +3990,19 @@
       </c>
       <c r="E73" s="13">
         <f t="shared" ca="1" si="13"/>
-        <v>46025.90693287037</v>
+        <v>46025.910277777781</v>
       </c>
       <c r="F73" s="13">
         <f t="shared" ca="1" si="15"/>
-        <v>46025.90693287037</v>
+        <v>46025.910277777781</v>
       </c>
       <c r="G73" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46025.910844907405</v>
+        <v>46025.912291666667</v>
       </c>
       <c r="H73" s="18">
         <f t="shared" ca="1" si="14"/>
-        <v>5.37</v>
+        <v>2.5300000000000002</v>
       </c>
       <c r="I73" s="3" t="s">
         <v>4</v>
@@ -4018,8 +4021,9 @@
       <c r="B74" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C74" s="3" t="s">
-        <v>161</v>
+      <c r="C74" s="4" t="str">
+        <f>_xlfn.XLOOKUP(B74, Mapping!A:A, Mapping!B:B, "Not Found")</f>
+        <v>CCAR_FS_TRIGGER</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>19</v>
@@ -4059,7 +4063,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6585004A-CAAF-4F9A-A882-FDE5BA3CBCD0}">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.36328125" customWidth="1"/>
@@ -4267,34 +4271,42 @@
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+      <c r="A26" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B27" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>153</v>
-      </c>
-      <c r="B27" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B28" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>155</v>
-      </c>
-      <c r="B28" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B29" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>157</v>
-      </c>
-      <c r="B29" t="s">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B30" t="s">
         <v>158</v>
       </c>
     </row>

</xml_diff>